<commit_message>
corpus(seep): re-emit reservoir-series files under the 'reservoir' type; build SEEPW-T07
Reservoir-drawdown/fill series blocks switch to kind='reservoir' so they keep the
submerged-only behavior under the new type split (gw017/018/019, gs2_rdd_inst/slow,
gs2_pond, VP102-t drawdown solve, and the RS2-67 field-diff tool); gw020 and gs2_heap
are rebuilt for the dropdown. All re-emitted .xlsx round-trip the kind correctly and
the 34 transient locks are unchanged.

SEEPW-T07 (multistep outflow) is un-parked: its stepped-suction base is now a plain
'head' series, so the negative-pressure Dirichlet is applied faithfully instead of
being dropped to the old uniform-H=0 field. gs2_mso built and locked at XSLOPE's own
solved heads; geostudio.md T07 flipped blocked -> built.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/verification/files/geostudio/gs2_heap.xlsx
+++ b/docs/verification/files/geostudio/gs2_heap.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="266">
   <si>
     <t>X</t>
   </si>
@@ -1023,6 +1023,9 @@
   </si>
   <si>
     <t>save_times</t>
+  </si>
+  <si>
+    <t>reservoir</t>
   </si>
 </sst>
 </file>
@@ -13843,7 +13846,9 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-      <c r="T6" s="1"/>
+      <c r="T6" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="U6" s="9"/>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
@@ -14109,7 +14114,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{21F200C9-4829-4345-9958-0F754F272AD0}">
-      <formula1>$T$4:$T$5</formula1>
+      <formula1>$T$4:$T$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14259,6 +14264,9 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
+      <c r="T6" s="1" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
@@ -14523,7 +14531,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{68C61D93-1721-F843-8E53-0F0E50006C65}">
-      <formula1>$T$4:$T$5</formula1>
+      <formula1>$T$4:$T$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
verification(SEEPW-T05): the ore column's van Genuchten pair is fit to the vendor conductivity table
The heap-leach example ships a retention spline and a conductivity spline for
the ore as independent 20-point curves, and xslope carries one (alpha, n) per
material. The pair now follows the standing rule for a vendor table against a
two-parameter law: least squares in log10 kr against the CONDUCTIVITY table,
over the suction range the run reaches. The column lives between psi = 0 and
the unit-gradient plateau the irrigation rate sets, with 0.785 m the largest
suction anywhere in the mesh over the march, so the fit is made over
psi <= 0.8 m and reads alpha = 1.3642 /m, n = 1.9888 -- 0.0009 decades rms
against the table there, where the retention pair reads 0.030.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/geostudio/gs2_heap.xlsx
+++ b/docs/verification/files/geostudio/gs2_heap.xlsx
@@ -6866,10 +6866,10 @@
         <v>-0.4</v>
       </c>
       <c r="AM11" s="3">
-        <v>1.3927</v>
+        <v>1.3642</v>
       </c>
       <c r="AN11" s="3">
-        <v>1.8965</v>
+        <v>1.9888</v>
       </c>
       <c r="AO11" s="3">
         <v>0.0001</v>
@@ -8312,9 +8312,7 @@
       <c r="A2" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="3">
-        <v>0</v>
-      </c>
+      <c r="B2" s="3"/>
       <c r="D2" s="24" t="s">
         <v>147</v>
       </c>

</xml_diff>